<commit_message>
update readme + guide de codage
</commit_message>
<xml_diff>
--- a/Peru_viral.xlsx
+++ b/Peru_viral.xlsx
@@ -121,21 +121,21 @@
     <t>text</t>
   </si>
   <si>
+    <t>E_D</t>
+  </si>
+  <si>
+    <t>Endorsement</t>
+  </si>
+  <si>
+    <t>Denuncia</t>
+  </si>
+  <si>
     <t>Eval</t>
   </si>
   <si>
     <t>Personal</t>
   </si>
   <si>
-    <t>E_D</t>
-  </si>
-  <si>
-    <t>Endorsement</t>
-  </si>
-  <si>
-    <t>Denuncia</t>
-  </si>
-  <si>
     <t>Pol_pub</t>
   </si>
   <si>
@@ -172,7 +172,7 @@
     <t>Tipo de actor</t>
   </si>
   <si>
-    <t>Posicionamiento de actor</t>
+    <t>General position</t>
   </si>
   <si>
     <t>NA</t>
@@ -2797,7 +2797,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -2824,6 +2824,10 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -2866,7 +2870,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2910,6 +2914,9 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -2918,7 +2925,7 @@
     <xf borderId="0" fillId="2" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -2933,7 +2940,7 @@
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -3438,17 +3445,17 @@
       <c r="AK2" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="AL2" s="10"/>
-      <c r="AM2" s="10"/>
+      <c r="AL2" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM2" s="10" t="s">
+        <v>67</v>
+      </c>
       <c r="AN2" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO2" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP2" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AO2" s="10"/>
+      <c r="AP2" s="10"/>
       <c r="AQ2" s="10"/>
       <c r="AR2" s="10"/>
       <c r="AS2" s="10"/>
@@ -3596,17 +3603,17 @@
       <c r="AK3" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="AL3" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM3" s="9" t="s">
+      <c r="AL3" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM3" s="9"/>
+      <c r="AN3" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN3" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO3" s="9"/>
-      <c r="AP3" s="10" t="s">
+      <c r="AO3" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP3" s="9" t="s">
         <v>68</v>
       </c>
       <c r="AQ3" s="9"/>
@@ -3755,15 +3762,15 @@
       <c r="AK4" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="AL4" s="10"/>
+      <c r="AL4" s="10" t="s">
+        <v>83</v>
+      </c>
       <c r="AM4" s="10"/>
       <c r="AN4" s="10" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="AO4" s="10"/>
-      <c r="AP4" s="10" t="s">
-        <v>68</v>
-      </c>
+      <c r="AP4" s="10"/>
       <c r="AQ4" s="10"/>
       <c r="AR4" s="10"/>
       <c r="AS4" s="10"/>
@@ -4063,15 +4070,15 @@
       <c r="AK6" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="AL6" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM6" s="10" t="s">
+      <c r="AL6" s="10"/>
+      <c r="AM6" s="10"/>
+      <c r="AN6" s="10"/>
+      <c r="AO6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP6" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN6" s="10"/>
-      <c r="AO6" s="10"/>
-      <c r="AP6" s="10"/>
       <c r="AQ6" s="10"/>
       <c r="AR6" s="10" t="s">
         <v>115</v>
@@ -4219,15 +4226,15 @@
       <c r="AK7" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="AL7" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM7" s="10" t="s">
+      <c r="AL7" s="10"/>
+      <c r="AM7" s="10"/>
+      <c r="AN7" s="10"/>
+      <c r="AO7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP7" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN7" s="10"/>
-      <c r="AO7" s="10"/>
-      <c r="AP7" s="10"/>
       <c r="AQ7" s="10"/>
       <c r="AR7" s="10" t="s">
         <v>115</v>
@@ -4375,15 +4382,15 @@
       <c r="AK8" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="AL8" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM8" s="10" t="s">
+      <c r="AL8" s="10"/>
+      <c r="AM8" s="10"/>
+      <c r="AN8" s="10"/>
+      <c r="AO8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP8" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN8" s="10"/>
-      <c r="AO8" s="10"/>
-      <c r="AP8" s="10"/>
       <c r="AQ8" s="10"/>
       <c r="AR8" s="10" t="s">
         <v>136</v>
@@ -4535,12 +4542,12 @@
       <c r="AK9" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="AL9" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL9" s="10"/>
       <c r="AM9" s="10"/>
       <c r="AN9" s="10"/>
-      <c r="AO9" s="10"/>
+      <c r="AO9" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP9" s="10"/>
       <c r="AQ9" s="10" t="s">
         <v>146</v>
@@ -4693,15 +4700,15 @@
       <c r="AK10" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="AL10" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM10" s="10" t="s">
+      <c r="AL10" s="10"/>
+      <c r="AM10" s="10"/>
+      <c r="AN10" s="10"/>
+      <c r="AO10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP10" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN10" s="10"/>
-      <c r="AO10" s="10"/>
-      <c r="AP10" s="10"/>
       <c r="AQ10" s="10"/>
       <c r="AR10" s="10" t="s">
         <v>136</v>
@@ -4851,15 +4858,15 @@
       <c r="AK11" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="AL11" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM11" s="10" t="s">
+      <c r="AL11" s="10"/>
+      <c r="AM11" s="10"/>
+      <c r="AN11" s="10"/>
+      <c r="AO11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP11" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN11" s="10"/>
-      <c r="AO11" s="10"/>
-      <c r="AP11" s="10"/>
       <c r="AQ11" s="10"/>
       <c r="AR11" s="10" t="s">
         <v>136</v>
@@ -5009,15 +5016,15 @@
       <c r="AK12" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="AL12" s="10"/>
+      <c r="AL12" s="10" t="s">
+        <v>83</v>
+      </c>
       <c r="AM12" s="10"/>
       <c r="AN12" s="10" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="AO12" s="10"/>
-      <c r="AP12" s="10" t="s">
-        <v>68</v>
-      </c>
+      <c r="AP12" s="10"/>
       <c r="AQ12" s="10"/>
       <c r="AR12" s="10"/>
       <c r="AS12" s="10"/>
@@ -5165,17 +5172,17 @@
       <c r="AK13" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="AL13" s="4" t="s">
-        <v>41</v>
+      <c r="AL13" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="AM13" s="10"/>
       <c r="AN13" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO13" s="10"/>
-      <c r="AP13" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AO13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP13" s="10"/>
       <c r="AQ13" s="10" t="s">
         <v>180</v>
       </c>
@@ -5327,17 +5334,17 @@
       <c r="AK14" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="AL14" s="4" t="s">
-        <v>41</v>
+      <c r="AL14" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="AM14" s="10"/>
       <c r="AN14" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO14" s="10"/>
-      <c r="AP14" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AO14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP14" s="10"/>
       <c r="AQ14" s="10" t="s">
         <v>190</v>
       </c>
@@ -5487,17 +5494,17 @@
       <c r="AK15" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="AL15" s="4" t="s">
-        <v>41</v>
+      <c r="AL15" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="AM15" s="10"/>
       <c r="AN15" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO15" s="10"/>
-      <c r="AP15" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AO15" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP15" s="10"/>
       <c r="AQ15" s="10" t="s">
         <v>199</v>
       </c>
@@ -5647,15 +5654,15 @@
       <c r="AK16" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="AL16" s="4" t="s">
+      <c r="AL16" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM16" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN16" s="10"/>
+      <c r="AO16" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="AM16" s="10"/>
-      <c r="AN16" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO16" s="10" t="s">
-        <v>67</v>
       </c>
       <c r="AP16" s="10"/>
       <c r="AQ16" s="10" t="s">
@@ -5809,12 +5816,12 @@
       <c r="AK17" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="AL17" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL17" s="10"/>
       <c r="AM17" s="10"/>
       <c r="AN17" s="10"/>
-      <c r="AO17" s="10"/>
+      <c r="AO17" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP17" s="10"/>
       <c r="AQ17" s="10" t="s">
         <v>190</v>
@@ -5965,14 +5972,14 @@
       <c r="AK18" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="AL18" s="10"/>
-      <c r="AM18" s="10"/>
-      <c r="AN18" s="10" t="s">
+      <c r="AL18" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO18" s="10" t="s">
+      <c r="AM18" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AN18" s="10"/>
+      <c r="AO18" s="10"/>
       <c r="AP18" s="10"/>
       <c r="AQ18" s="10"/>
       <c r="AR18" s="10"/>
@@ -6867,12 +6874,12 @@
       <c r="AK24" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="AL24" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL24" s="10"/>
       <c r="AM24" s="10"/>
       <c r="AN24" s="10"/>
-      <c r="AO24" s="10"/>
+      <c r="AO24" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP24" s="10"/>
       <c r="AQ24" s="10" t="s">
         <v>262</v>
@@ -7327,12 +7334,12 @@
       <c r="AK27" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="AL27" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL27" s="10"/>
       <c r="AM27" s="10"/>
       <c r="AN27" s="10"/>
-      <c r="AO27" s="10"/>
+      <c r="AO27" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP27" s="10"/>
       <c r="AQ27" s="10" t="s">
         <v>146</v>
@@ -7483,12 +7490,12 @@
       <c r="AK28" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="AL28" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL28" s="10"/>
       <c r="AM28" s="10"/>
       <c r="AN28" s="10"/>
-      <c r="AO28" s="10"/>
+      <c r="AO28" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP28" s="10"/>
       <c r="AQ28" s="10" t="s">
         <v>190</v>
@@ -7639,14 +7646,14 @@
       <c r="AK29" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="AL29" s="10"/>
-      <c r="AM29" s="10"/>
-      <c r="AN29" s="10" t="s">
+      <c r="AL29" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO29" s="10" t="s">
+      <c r="AM29" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AN29" s="10"/>
+      <c r="AO29" s="10"/>
       <c r="AP29" s="10"/>
       <c r="AQ29" s="10"/>
       <c r="AR29" s="10"/>
@@ -7943,12 +7950,12 @@
       <c r="AK31" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="AL31" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL31" s="10"/>
       <c r="AM31" s="10"/>
       <c r="AN31" s="10"/>
-      <c r="AO31" s="10"/>
+      <c r="AO31" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP31" s="10"/>
       <c r="AQ31" s="10" t="s">
         <v>190</v>
@@ -8551,12 +8558,12 @@
       <c r="AK35" s="9" t="s">
         <v>326</v>
       </c>
-      <c r="AL35" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL35" s="10"/>
       <c r="AM35" s="10"/>
       <c r="AN35" s="10"/>
-      <c r="AO35" s="10"/>
+      <c r="AO35" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP35" s="10"/>
       <c r="AQ35" s="10" t="s">
         <v>180</v>
@@ -8857,12 +8864,12 @@
       <c r="AK37" s="9" t="s">
         <v>340</v>
       </c>
-      <c r="AL37" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL37" s="10"/>
       <c r="AM37" s="10"/>
       <c r="AN37" s="10"/>
-      <c r="AO37" s="10"/>
+      <c r="AO37" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP37" s="10"/>
       <c r="AQ37" s="10" t="s">
         <v>180</v>
@@ -9313,10 +9320,10 @@
       <c r="AK40" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="AL40" s="4"/>
+      <c r="AL40" s="10"/>
       <c r="AM40" s="10"/>
       <c r="AN40" s="10"/>
-      <c r="AO40" s="10"/>
+      <c r="AO40" s="4"/>
       <c r="AP40" s="10"/>
       <c r="AQ40" s="10"/>
       <c r="AR40" s="10"/>
@@ -9463,14 +9470,14 @@
       <c r="AK41" s="9" t="s">
         <v>363</v>
       </c>
-      <c r="AL41" s="10"/>
-      <c r="AM41" s="10"/>
-      <c r="AN41" s="10" t="s">
+      <c r="AL41" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO41" s="10" t="s">
+      <c r="AM41" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AN41" s="10"/>
+      <c r="AO41" s="10"/>
       <c r="AP41" s="10"/>
       <c r="AQ41" s="10"/>
       <c r="AR41" s="10"/>
@@ -9617,12 +9624,12 @@
       <c r="AK42" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="AL42" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL42" s="10"/>
       <c r="AM42" s="10"/>
       <c r="AN42" s="10"/>
-      <c r="AO42" s="10"/>
+      <c r="AO42" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP42" s="10"/>
       <c r="AQ42" s="10" t="s">
         <v>180</v>
@@ -9773,14 +9780,14 @@
       <c r="AK43" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="AL43" s="10"/>
-      <c r="AM43" s="10"/>
-      <c r="AN43" s="10" t="s">
+      <c r="AL43" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO43" s="10" t="s">
+      <c r="AM43" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AN43" s="10"/>
+      <c r="AO43" s="10"/>
       <c r="AP43" s="10"/>
       <c r="AQ43" s="10"/>
       <c r="AR43" s="10"/>
@@ -9852,7 +9859,7 @@
       <c r="L44" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="M44" s="7" t="s">
+      <c r="M44" s="14" t="s">
         <v>374</v>
       </c>
       <c r="N44" s="6">
@@ -9927,15 +9934,15 @@
       <c r="AK44" s="9" t="s">
         <v>378</v>
       </c>
-      <c r="AL44" s="4" t="s">
+      <c r="AL44" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM44" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN44" s="10"/>
+      <c r="AO44" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="AM44" s="10"/>
-      <c r="AN44" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO44" s="10" t="s">
-        <v>67</v>
       </c>
       <c r="AP44" s="10"/>
       <c r="AQ44" s="10" t="s">
@@ -10087,16 +10094,16 @@
       <c r="AK45" s="9" t="s">
         <v>383</v>
       </c>
-      <c r="AL45" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM45" s="10" t="s">
+      <c r="AL45" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM45" s="10"/>
+      <c r="AN45" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN45" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO45" s="10"/>
+      <c r="AO45" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="AP45" s="10" t="s">
         <v>68</v>
       </c>
@@ -10109,7 +10116,7 @@
       <c r="AU45" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV45" s="14" t="s">
+      <c r="AV45" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW45" s="9" t="s">
@@ -10247,16 +10254,16 @@
       <c r="AK46" s="9" t="s">
         <v>393</v>
       </c>
-      <c r="AL46" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM46" s="10" t="s">
+      <c r="AL46" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM46" s="10"/>
+      <c r="AN46" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN46" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO46" s="10"/>
+      <c r="AO46" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="AP46" s="10" t="s">
         <v>67</v>
       </c>
@@ -10269,7 +10276,7 @@
       <c r="AU46" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV46" s="14" t="s">
+      <c r="AV46" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW46" s="9" t="s">
@@ -10405,17 +10412,17 @@
       <c r="AK47" s="9" t="s">
         <v>399</v>
       </c>
-      <c r="AL47" s="4" t="s">
+      <c r="AL47" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM47" s="10"/>
+      <c r="AN47" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO47" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AM47" s="10"/>
-      <c r="AN47" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO47" s="10"/>
-      <c r="AP47" s="10" t="s">
-        <v>68</v>
-      </c>
+      <c r="AP47" s="10"/>
       <c r="AQ47" s="10" t="s">
         <v>190</v>
       </c>
@@ -10427,7 +10434,7 @@
       <c r="AU47" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV47" s="14" t="s">
+      <c r="AV47" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW47" s="9" t="s">
@@ -10565,15 +10572,15 @@
       <c r="AK48" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="AL48" s="10"/>
+      <c r="AL48" s="5" t="s">
+        <v>83</v>
+      </c>
       <c r="AM48" s="10"/>
-      <c r="AN48" s="5" t="s">
-        <v>83</v>
+      <c r="AN48" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="AO48" s="10"/>
-      <c r="AP48" s="10" t="s">
-        <v>68</v>
-      </c>
+      <c r="AP48" s="10"/>
       <c r="AQ48" s="10"/>
       <c r="AR48" s="10"/>
       <c r="AS48" s="10"/>
@@ -10583,7 +10590,7 @@
       <c r="AU48" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV48" s="14" t="s">
+      <c r="AV48" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW48" s="9" t="s">
@@ -10721,20 +10728,20 @@
       <c r="AK49" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="AL49" s="4" t="s">
-        <v>37</v>
+      <c r="AL49" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="AM49" s="10" t="s">
         <v>67</v>
       </c>
       <c r="AN49" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO49" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO49" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP49" s="10" t="s">
         <v>67</v>
-      </c>
-      <c r="AP49" s="10" t="s">
-        <v>68</v>
       </c>
       <c r="AQ49" s="10"/>
       <c r="AR49" s="10"/>
@@ -10745,7 +10752,7 @@
       <c r="AU49" s="9">
         <v>2.0</v>
       </c>
-      <c r="AV49" s="14" t="s">
+      <c r="AV49" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW49" s="5" t="s">
@@ -10882,16 +10889,16 @@
       <c r="AK50" s="9" t="s">
         <v>426</v>
       </c>
-      <c r="AL50" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM50" s="10" t="s">
+      <c r="AL50" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM50" s="10"/>
+      <c r="AN50" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN50" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO50" s="10"/>
+      <c r="AO50" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="AP50" s="10" t="s">
         <v>67</v>
       </c>
@@ -10904,7 +10911,7 @@
       <c r="AU50" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV50" s="14" t="s">
+      <c r="AV50" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW50" s="9" t="s">
@@ -11040,15 +11047,15 @@
       <c r="AK51" s="9" t="s">
         <v>432</v>
       </c>
-      <c r="AL51" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM51" s="10" t="s">
+      <c r="AL51" s="10"/>
+      <c r="AM51" s="10"/>
+      <c r="AN51" s="10"/>
+      <c r="AO51" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP51" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN51" s="10"/>
-      <c r="AO51" s="10"/>
-      <c r="AP51" s="10"/>
       <c r="AQ51" s="10"/>
       <c r="AR51" s="10"/>
       <c r="AS51" s="10"/>
@@ -11058,7 +11065,7 @@
       <c r="AU51" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV51" s="14" t="s">
+      <c r="AV51" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW51" s="9" t="s">
@@ -11194,16 +11201,16 @@
       <c r="AK52" s="9" t="s">
         <v>439</v>
       </c>
-      <c r="AL52" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM52" s="10" t="s">
+      <c r="AL52" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM52" s="10"/>
+      <c r="AN52" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN52" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO52" s="10"/>
+      <c r="AO52" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="AP52" s="10" t="s">
         <v>68</v>
       </c>
@@ -11216,7 +11223,7 @@
       <c r="AU52" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV52" s="14" t="s">
+      <c r="AV52" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW52" s="9" t="s">
@@ -11352,16 +11359,16 @@
       <c r="AK53" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="AL53" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM53" s="10" t="s">
+      <c r="AL53" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM53" s="10"/>
+      <c r="AN53" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN53" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO53" s="10"/>
+      <c r="AO53" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="AP53" s="10" t="s">
         <v>67</v>
       </c>
@@ -11374,7 +11381,7 @@
       <c r="AU53" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV53" s="14" t="s">
+      <c r="AV53" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW53" s="9" t="s">
@@ -11512,14 +11519,14 @@
       <c r="AK54" s="9" t="s">
         <v>452</v>
       </c>
-      <c r="AL54" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM54" s="10" t="s">
+      <c r="AM54" s="10"/>
+      <c r="AN54" s="10"/>
+      <c r="AO54" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP54" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AO54" s="10"/>
-      <c r="AP54" s="10"/>
       <c r="AQ54" s="10"/>
       <c r="AR54" s="10"/>
       <c r="AS54" s="10"/>
@@ -11529,7 +11536,7 @@
       <c r="AU54" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV54" s="14" t="s">
+      <c r="AV54" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW54" s="9" t="s">
@@ -11665,17 +11672,17 @@
       <c r="AK55" s="9" t="s">
         <v>459</v>
       </c>
-      <c r="AL55" s="4" t="s">
+      <c r="AL55" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM55" s="10"/>
+      <c r="AN55" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO55" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AM55" s="10"/>
-      <c r="AN55" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO55" s="10"/>
-      <c r="AP55" s="10" t="s">
-        <v>67</v>
-      </c>
+      <c r="AP55" s="10"/>
       <c r="AQ55" s="10" t="s">
         <v>190</v>
       </c>
@@ -11689,7 +11696,7 @@
       <c r="AU55" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV55" s="14" t="s">
+      <c r="AV55" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW55" s="9" t="s">
@@ -11827,15 +11834,15 @@
       <c r="AK56" s="9" t="s">
         <v>466</v>
       </c>
-      <c r="AL56" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM56" s="10" t="s">
+      <c r="AL56" s="10"/>
+      <c r="AM56" s="10"/>
+      <c r="AN56" s="10"/>
+      <c r="AO56" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP56" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN56" s="10"/>
-      <c r="AO56" s="10"/>
-      <c r="AP56" s="10"/>
       <c r="AQ56" s="10"/>
       <c r="AR56" s="10" t="s">
         <v>115</v>
@@ -11847,7 +11854,7 @@
       <c r="AU56" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV56" s="14" t="s">
+      <c r="AV56" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW56" s="9" t="s">
@@ -11997,7 +12004,7 @@
       <c r="AU57" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV57" s="14" t="s">
+      <c r="AV57" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW57" s="9" t="s">
@@ -12133,15 +12140,15 @@
       <c r="AK58" s="9" t="s">
         <v>476</v>
       </c>
-      <c r="AL58" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM58" s="10" t="s">
+      <c r="AL58" s="10"/>
+      <c r="AM58" s="10"/>
+      <c r="AN58" s="10"/>
+      <c r="AO58" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP58" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN58" s="10"/>
-      <c r="AO58" s="10"/>
-      <c r="AP58" s="10"/>
       <c r="AQ58" s="10"/>
       <c r="AR58" s="10"/>
       <c r="AS58" s="10"/>
@@ -12151,7 +12158,7 @@
       <c r="AU58" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV58" s="14" t="s">
+      <c r="AV58" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW58" s="9" t="s">
@@ -12301,7 +12308,7 @@
       <c r="AU59" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV59" s="14" t="s">
+      <c r="AV59" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW59" s="9" t="s">
@@ -12453,7 +12460,7 @@
       <c r="AU60" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV60" s="14" t="s">
+      <c r="AV60" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW60" s="9" t="s">
@@ -12591,15 +12598,15 @@
       <c r="AK61" s="9" t="s">
         <v>495</v>
       </c>
-      <c r="AL61" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM61" s="10" t="s">
+      <c r="AL61" s="10"/>
+      <c r="AM61" s="10"/>
+      <c r="AN61" s="10"/>
+      <c r="AO61" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP61" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN61" s="10"/>
-      <c r="AO61" s="10"/>
-      <c r="AP61" s="10"/>
       <c r="AQ61" s="10"/>
       <c r="AR61" s="10"/>
       <c r="AS61" s="10"/>
@@ -12609,7 +12616,7 @@
       <c r="AU61" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV61" s="14" t="s">
+      <c r="AV61" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW61" s="9" t="s">
@@ -12745,12 +12752,12 @@
       <c r="AK62" s="9" t="s">
         <v>499</v>
       </c>
-      <c r="AL62" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL62" s="10"/>
       <c r="AM62" s="10"/>
       <c r="AN62" s="10"/>
-      <c r="AO62" s="10"/>
+      <c r="AO62" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP62" s="10"/>
       <c r="AQ62" s="10" t="s">
         <v>180</v>
@@ -12765,7 +12772,7 @@
       <c r="AU62" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV62" s="14" t="s">
+      <c r="AV62" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW62" s="9" t="s">
@@ -12903,16 +12910,16 @@
       <c r="AK63" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="AL63" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM63" s="10" t="s">
+      <c r="AL63" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM63" s="10"/>
+      <c r="AN63" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN63" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO63" s="10"/>
+      <c r="AO63" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="AP63" s="10" t="s">
         <v>68</v>
       </c>
@@ -12925,7 +12932,7 @@
       <c r="AU63" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV63" s="14" t="s">
+      <c r="AV63" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW63" s="9" t="s">
@@ -13061,12 +13068,12 @@
       <c r="AK64" s="9" t="s">
         <v>512</v>
       </c>
-      <c r="AL64" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL64" s="10"/>
       <c r="AM64" s="10"/>
       <c r="AN64" s="10"/>
-      <c r="AO64" s="10"/>
+      <c r="AO64" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP64" s="10"/>
       <c r="AQ64" s="10" t="s">
         <v>513</v>
@@ -13081,7 +13088,7 @@
       <c r="AU64" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV64" s="14" t="s">
+      <c r="AV64" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW64" s="9" t="s">
@@ -13231,7 +13238,7 @@
       <c r="AU65" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV65" s="14" t="s">
+      <c r="AV65" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW65" s="9" t="s">
@@ -13369,15 +13376,15 @@
       <c r="AK66" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="AL66" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM66" s="10" t="s">
+      <c r="AL66" s="10"/>
+      <c r="AM66" s="10"/>
+      <c r="AN66" s="10"/>
+      <c r="AO66" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP66" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN66" s="10"/>
-      <c r="AO66" s="10"/>
-      <c r="AP66" s="10"/>
       <c r="AQ66" s="10"/>
       <c r="AR66" s="10" t="s">
         <v>115</v>
@@ -13389,7 +13396,7 @@
       <c r="AU66" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV66" s="14" t="s">
+      <c r="AV66" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW66" s="9" t="s">
@@ -13525,12 +13532,12 @@
       <c r="AK67" s="9" t="s">
         <v>528</v>
       </c>
-      <c r="AL67" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL67" s="10"/>
       <c r="AM67" s="10"/>
       <c r="AN67" s="10"/>
-      <c r="AO67" s="10"/>
+      <c r="AO67" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP67" s="10"/>
       <c r="AQ67" s="10" t="s">
         <v>529</v>
@@ -13545,7 +13552,7 @@
       <c r="AU67" s="10">
         <v>2.0</v>
       </c>
-      <c r="AV67" s="14" t="s">
+      <c r="AV67" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW67" s="9" t="s">
@@ -13697,7 +13704,7 @@
       <c r="AU68" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV68" s="14" t="s">
+      <c r="AV68" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW68" s="9" t="s">
@@ -13847,7 +13854,7 @@
       <c r="AU69" s="10">
         <v>0.0</v>
       </c>
-      <c r="AV69" s="14" t="s">
+      <c r="AV69" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW69" s="9" t="s">
@@ -13983,17 +13990,17 @@
       <c r="AK70" s="9" t="s">
         <v>550</v>
       </c>
-      <c r="AL70" s="4" t="s">
+      <c r="AL70" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM70" s="10"/>
+      <c r="AN70" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO70" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AM70" s="10"/>
-      <c r="AN70" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO70" s="10"/>
-      <c r="AP70" s="10" t="s">
-        <v>68</v>
-      </c>
+      <c r="AP70" s="10"/>
       <c r="AQ70" s="10" t="s">
         <v>190</v>
       </c>
@@ -14007,7 +14014,7 @@
       <c r="AU70" s="10">
         <v>1.0</v>
       </c>
-      <c r="AV70" s="14" t="s">
+      <c r="AV70" s="15" t="s">
         <v>384</v>
       </c>
       <c r="AW70" s="9" t="s">
@@ -14295,19 +14302,19 @@
       <c r="AK72" s="9" t="s">
         <v>568</v>
       </c>
-      <c r="AL72" s="4" t="s">
+      <c r="AL72" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM72" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN72" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO72" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AM72" s="10"/>
-      <c r="AN72" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO72" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="AP72" s="10" t="s">
-        <v>67</v>
-      </c>
+      <c r="AP72" s="10"/>
       <c r="AQ72" s="10" t="s">
         <v>180</v>
       </c>
@@ -14459,15 +14466,15 @@
       <c r="AK73" s="9" t="s">
         <v>574</v>
       </c>
-      <c r="AL73" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM73" s="10" t="s">
+      <c r="AL73" s="10"/>
+      <c r="AM73" s="10"/>
+      <c r="AN73" s="10"/>
+      <c r="AO73" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP73" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN73" s="10"/>
-      <c r="AO73" s="10"/>
-      <c r="AP73" s="10"/>
       <c r="AQ73" s="10"/>
       <c r="AR73" s="10" t="s">
         <v>115</v>
@@ -14919,14 +14926,14 @@
       <c r="AK76" s="9" t="s">
         <v>587</v>
       </c>
-      <c r="AL76" s="4"/>
-      <c r="AM76" s="10"/>
-      <c r="AN76" s="10" t="s">
+      <c r="AL76" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO76" s="10" t="s">
+      <c r="AM76" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AN76" s="10"/>
+      <c r="AO76" s="4"/>
       <c r="AP76" s="10"/>
       <c r="AQ76" s="10"/>
       <c r="AR76" s="10"/>
@@ -15071,17 +15078,17 @@
       <c r="AK77" s="9" t="s">
         <v>593</v>
       </c>
-      <c r="AL77" s="4" t="s">
+      <c r="AL77" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AM77" s="10"/>
+      <c r="AN77" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO77" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AM77" s="10"/>
-      <c r="AN77" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO77" s="10"/>
-      <c r="AP77" s="10" t="s">
-        <v>68</v>
-      </c>
+      <c r="AP77" s="10"/>
       <c r="AQ77" s="10" t="s">
         <v>529</v>
       </c>
@@ -15233,14 +15240,14 @@
       <c r="AK78" s="9" t="s">
         <v>601</v>
       </c>
-      <c r="AL78" s="10"/>
-      <c r="AM78" s="10"/>
-      <c r="AN78" s="5" t="s">
+      <c r="AL78" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="AO78" s="10" t="s">
+      <c r="AM78" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AN78" s="10"/>
+      <c r="AO78" s="10"/>
       <c r="AP78" s="10"/>
       <c r="AQ78" s="10"/>
       <c r="AR78" s="10"/>
@@ -15387,19 +15394,19 @@
       <c r="AK79" s="9" t="s">
         <v>607</v>
       </c>
-      <c r="AL79" s="4" t="s">
-        <v>37</v>
+      <c r="AL79" s="10" t="s">
+        <v>66</v>
       </c>
       <c r="AM79" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN79" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO79" s="10" t="s">
+      <c r="AN79" s="10"/>
+      <c r="AO79" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP79" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AP79" s="10"/>
       <c r="AQ79" s="10"/>
       <c r="AR79" s="10"/>
       <c r="AS79" s="10"/>
@@ -15545,14 +15552,14 @@
       <c r="AK80" s="9" t="s">
         <v>611</v>
       </c>
-      <c r="AL80" s="10"/>
-      <c r="AM80" s="10"/>
-      <c r="AN80" s="10" t="s">
+      <c r="AL80" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO80" s="10" t="s">
+      <c r="AM80" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AN80" s="10"/>
+      <c r="AO80" s="10"/>
       <c r="AP80" s="10"/>
       <c r="AQ80" s="10"/>
       <c r="AR80" s="10"/>
@@ -15851,14 +15858,14 @@
       <c r="AK82" s="9" t="s">
         <v>625</v>
       </c>
-      <c r="AL82" s="4"/>
-      <c r="AM82" s="10"/>
-      <c r="AN82" s="10" t="s">
+      <c r="AL82" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO82" s="10" t="s">
+      <c r="AM82" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AN82" s="10"/>
+      <c r="AO82" s="4"/>
       <c r="AP82" s="10"/>
       <c r="AQ82" s="10"/>
       <c r="AR82" s="10"/>
@@ -16005,14 +16012,14 @@
       <c r="AK83" s="9" t="s">
         <v>632</v>
       </c>
-      <c r="AL83" s="4"/>
-      <c r="AM83" s="10"/>
-      <c r="AN83" s="10" t="s">
+      <c r="AL83" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO83" s="10" t="s">
+      <c r="AM83" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AN83" s="10"/>
+      <c r="AO83" s="4"/>
       <c r="AP83" s="10"/>
       <c r="AQ83" s="10"/>
       <c r="AR83" s="10"/>
@@ -16159,19 +16166,19 @@
       <c r="AK84" s="9" t="s">
         <v>636</v>
       </c>
-      <c r="AL84" s="4" t="s">
-        <v>37</v>
+      <c r="AL84" s="10" t="s">
+        <v>66</v>
       </c>
       <c r="AM84" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN84" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO84" s="10" t="s">
+      <c r="AN84" s="10"/>
+      <c r="AO84" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP84" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AP84" s="10"/>
       <c r="AQ84" s="10"/>
       <c r="AR84" s="10"/>
       <c r="AS84" s="10"/>
@@ -16317,19 +16324,19 @@
       <c r="AK85" s="9" t="s">
         <v>643</v>
       </c>
-      <c r="AL85" s="4" t="s">
-        <v>37</v>
+      <c r="AL85" s="10" t="s">
+        <v>66</v>
       </c>
       <c r="AM85" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN85" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO85" s="10" t="s">
+      <c r="AN85" s="10"/>
+      <c r="AO85" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP85" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AP85" s="10"/>
       <c r="AQ85" s="10"/>
       <c r="AR85" s="10"/>
       <c r="AS85" s="10"/>
@@ -16475,14 +16482,14 @@
       <c r="AK86" s="9" t="s">
         <v>648</v>
       </c>
-      <c r="AL86" s="10"/>
-      <c r="AM86" s="10"/>
-      <c r="AN86" s="10" t="s">
+      <c r="AL86" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO86" s="10" t="s">
+      <c r="AM86" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AN86" s="10"/>
+      <c r="AO86" s="10"/>
       <c r="AP86" s="10"/>
       <c r="AQ86" s="10"/>
       <c r="AR86" s="10"/>
@@ -16629,14 +16636,14 @@
       <c r="AK87" s="9" t="s">
         <v>655</v>
       </c>
-      <c r="AL87" s="10"/>
-      <c r="AM87" s="10"/>
-      <c r="AN87" s="10" t="s">
+      <c r="AL87" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO87" s="10" t="s">
+      <c r="AM87" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AN87" s="10"/>
+      <c r="AO87" s="10"/>
       <c r="AP87" s="10"/>
       <c r="AQ87" s="10"/>
       <c r="AR87" s="10"/>
@@ -16933,12 +16940,12 @@
       <c r="AK89" s="9" t="s">
         <v>664</v>
       </c>
-      <c r="AL89" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL89" s="10"/>
       <c r="AM89" s="10"/>
       <c r="AN89" s="10"/>
-      <c r="AO89" s="10"/>
+      <c r="AO89" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP89" s="10"/>
       <c r="AQ89" s="10" t="s">
         <v>665</v>
@@ -17089,17 +17096,17 @@
       <c r="AK90" s="9" t="s">
         <v>668</v>
       </c>
-      <c r="AL90" s="10"/>
-      <c r="AM90" s="10"/>
+      <c r="AL90" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM90" s="10" t="s">
+        <v>68</v>
+      </c>
       <c r="AN90" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO90" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="AP90" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AO90" s="10"/>
+      <c r="AP90" s="10"/>
       <c r="AQ90" s="10"/>
       <c r="AR90" s="10"/>
       <c r="AS90" s="10"/>
@@ -17245,15 +17252,15 @@
       <c r="AK91" s="9" t="s">
         <v>672</v>
       </c>
-      <c r="AL91" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM91" s="10" t="s">
+      <c r="AL91" s="10"/>
+      <c r="AM91" s="10"/>
+      <c r="AN91" s="10"/>
+      <c r="AO91" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP91" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN91" s="10"/>
-      <c r="AO91" s="10"/>
-      <c r="AP91" s="10"/>
       <c r="AQ91" s="10"/>
       <c r="AR91" s="10"/>
       <c r="AS91" s="10"/>
@@ -17399,12 +17406,12 @@
       <c r="AK92" s="9" t="s">
         <v>678</v>
       </c>
-      <c r="AL92" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL92" s="10"/>
       <c r="AM92" s="10"/>
       <c r="AN92" s="10"/>
-      <c r="AO92" s="10"/>
+      <c r="AO92" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP92" s="10"/>
       <c r="AQ92" s="10" t="s">
         <v>665</v>
@@ -17555,12 +17562,12 @@
       <c r="AK93" s="9" t="s">
         <v>683</v>
       </c>
-      <c r="AL93" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="AL93" s="10"/>
       <c r="AM93" s="10"/>
       <c r="AN93" s="10"/>
-      <c r="AO93" s="10"/>
+      <c r="AO93" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="AP93" s="10"/>
       <c r="AQ93" s="10" t="s">
         <v>372</v>
@@ -17711,14 +17718,14 @@
       <c r="AK94" s="9" t="s">
         <v>690</v>
       </c>
-      <c r="AL94" s="10"/>
-      <c r="AM94" s="10"/>
-      <c r="AN94" s="10" t="s">
+      <c r="AL94" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO94" s="10" t="s">
+      <c r="AM94" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AN94" s="10"/>
+      <c r="AO94" s="10"/>
       <c r="AP94" s="10"/>
       <c r="AQ94" s="10"/>
       <c r="AR94" s="10"/>
@@ -17867,15 +17874,15 @@
       <c r="AK95" s="9" t="s">
         <v>699</v>
       </c>
-      <c r="AL95" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM95" s="10" t="s">
+      <c r="AL95" s="10"/>
+      <c r="AM95" s="10"/>
+      <c r="AN95" s="10"/>
+      <c r="AO95" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP95" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN95" s="10"/>
-      <c r="AO95" s="10"/>
-      <c r="AP95" s="10"/>
       <c r="AQ95" s="10"/>
       <c r="AR95" s="10" t="s">
         <v>115</v>
@@ -18023,14 +18030,14 @@
       <c r="AK96" s="9" t="s">
         <v>708</v>
       </c>
-      <c r="AL96" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM96" s="10" t="s">
+      <c r="AL96" s="10"/>
+      <c r="AM96" s="10"/>
+      <c r="AN96" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN96" s="10"/>
-      <c r="AO96" s="10"/>
+      <c r="AO96" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="AP96" s="10" t="s">
         <v>68</v>
       </c>
@@ -18329,19 +18336,19 @@
       <c r="AK98" s="9" t="s">
         <v>719</v>
       </c>
-      <c r="AL98" s="4" t="s">
-        <v>37</v>
+      <c r="AL98" s="10" t="s">
+        <v>66</v>
       </c>
       <c r="AM98" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN98" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO98" s="10" t="s">
+      <c r="AN98" s="10"/>
+      <c r="AO98" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP98" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AP98" s="10"/>
       <c r="AQ98" s="10"/>
       <c r="AR98" s="10"/>
       <c r="AS98" s="10"/>
@@ -18637,19 +18644,19 @@
       <c r="AK100" s="9" t="s">
         <v>732</v>
       </c>
-      <c r="AL100" s="4" t="s">
-        <v>37</v>
+      <c r="AL100" s="10" t="s">
+        <v>66</v>
       </c>
       <c r="AM100" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN100" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO100" s="10" t="s">
+      <c r="AN100" s="10"/>
+      <c r="AO100" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP100" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AP100" s="10"/>
       <c r="AQ100" s="10"/>
       <c r="AR100" s="10"/>
       <c r="AS100" s="10"/>
@@ -18795,14 +18802,14 @@
       <c r="AK101" s="9" t="s">
         <v>740</v>
       </c>
-      <c r="AL101" s="10"/>
-      <c r="AM101" s="10"/>
-      <c r="AN101" s="10" t="s">
+      <c r="AL101" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO101" s="10" t="s">
+      <c r="AM101" s="10" t="s">
         <v>68</v>
       </c>
+      <c r="AN101" s="10"/>
+      <c r="AO101" s="10"/>
       <c r="AP101" s="10"/>
       <c r="AQ101" s="10"/>
       <c r="AR101" s="10"/>
@@ -19097,15 +19104,15 @@
       <c r="AK103" s="9" t="s">
         <v>750</v>
       </c>
-      <c r="AL103" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM103" s="10" t="s">
+      <c r="AL103" s="10"/>
+      <c r="AM103" s="10"/>
+      <c r="AN103" s="10"/>
+      <c r="AO103" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP103" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN103" s="10"/>
-      <c r="AO103" s="10"/>
-      <c r="AP103" s="10"/>
       <c r="AQ103" s="10"/>
       <c r="AR103" s="10"/>
       <c r="AS103" s="10" t="s">
@@ -19253,15 +19260,15 @@
       <c r="AK104" s="9" t="s">
         <v>754</v>
       </c>
-      <c r="AL104" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM104" s="10" t="s">
+      <c r="AL104" s="10"/>
+      <c r="AM104" s="10"/>
+      <c r="AN104" s="10"/>
+      <c r="AO104" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP104" s="10" t="s">
         <v>755</v>
       </c>
-      <c r="AN104" s="10"/>
-      <c r="AO104" s="10"/>
-      <c r="AP104" s="10"/>
       <c r="AQ104" s="10"/>
       <c r="AR104" s="10" t="s">
         <v>136</v>
@@ -19409,15 +19416,15 @@
       <c r="AK105" s="9" t="s">
         <v>761</v>
       </c>
-      <c r="AL105" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM105" s="10" t="s">
+      <c r="AL105" s="10"/>
+      <c r="AM105" s="10"/>
+      <c r="AN105" s="10"/>
+      <c r="AO105" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP105" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AN105" s="10"/>
-      <c r="AO105" s="10"/>
-      <c r="AP105" s="10"/>
       <c r="AQ105" s="10"/>
       <c r="AR105" s="10"/>
       <c r="AS105" s="10"/>
@@ -19563,14 +19570,14 @@
       <c r="AK106" s="9" t="s">
         <v>765</v>
       </c>
-      <c r="AL106" s="10"/>
-      <c r="AM106" s="10"/>
-      <c r="AN106" s="10" t="s">
+      <c r="AL106" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AO106" s="10" t="s">
+      <c r="AM106" s="10" t="s">
         <v>67</v>
       </c>
+      <c r="AN106" s="10"/>
+      <c r="AO106" s="10"/>
       <c r="AP106" s="10"/>
       <c r="AQ106" s="10"/>
       <c r="AR106" s="10"/>
@@ -19717,15 +19724,15 @@
       <c r="AK107" s="9" t="s">
         <v>769</v>
       </c>
-      <c r="AL107" s="4" t="s">
+      <c r="AL107" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM107" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN107" s="10"/>
+      <c r="AO107" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="AM107" s="10"/>
-      <c r="AN107" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO107" s="10" t="s">
-        <v>67</v>
       </c>
       <c r="AP107" s="10"/>
       <c r="AQ107" s="10" t="s">
@@ -19877,19 +19884,19 @@
       <c r="AK108" s="9" t="s">
         <v>774</v>
       </c>
-      <c r="AL108" s="4" t="s">
-        <v>37</v>
+      <c r="AL108" s="10" t="s">
+        <v>66</v>
       </c>
       <c r="AM108" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN108" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO108" s="10" t="s">
+      <c r="AN108" s="10"/>
+      <c r="AO108" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP108" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AP108" s="10"/>
       <c r="AQ108" s="10"/>
       <c r="AR108" s="10"/>
       <c r="AS108" s="10"/>
@@ -20037,15 +20044,15 @@
       <c r="AK109" s="9" t="s">
         <v>779</v>
       </c>
-      <c r="AL109" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM109" s="10" t="s">
+      <c r="AL109" s="10"/>
+      <c r="AM109" s="10"/>
+      <c r="AN109" s="10"/>
+      <c r="AO109" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP109" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AN109" s="10"/>
-      <c r="AO109" s="10"/>
-      <c r="AP109" s="10"/>
       <c r="AQ109" s="10"/>
       <c r="AR109" s="10"/>
       <c r="AS109" s="10"/>
@@ -20080,1588 +20087,1588 @@
       <c r="BD109" s="11"/>
     </row>
     <row r="110">
-      <c r="A110" s="15">
+      <c r="A110" s="16">
         <v>34.0</v>
       </c>
-      <c r="B110" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C110" s="15" t="s">
+      <c r="B110" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C110" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D110" s="16">
+      <c r="D110" s="17">
         <v>46174.00927083333</v>
       </c>
-      <c r="E110" s="15" t="s">
+      <c r="E110" s="16" t="s">
         <v>781</v>
       </c>
-      <c r="F110" s="15" t="b">
+      <c r="F110" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G110" s="15" t="s">
+      <c r="G110" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H110" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I110" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J110" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K110" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L110" s="15" t="s">
+      <c r="H110" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I110" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J110" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K110" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L110" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M110" s="17" t="s">
+      <c r="M110" s="18" t="s">
         <v>782</v>
       </c>
-      <c r="N110" s="16">
+      <c r="N110" s="17">
         <v>46177.13055555556</v>
       </c>
-      <c r="O110" s="15" t="s">
+      <c r="O110" s="16" t="s">
         <v>783</v>
       </c>
-      <c r="P110" s="15" t="s">
+      <c r="P110" s="16" t="s">
         <v>784</v>
       </c>
-      <c r="Q110" s="15" t="s">
+      <c r="Q110" s="16" t="s">
         <v>785</v>
       </c>
-      <c r="R110" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S110" s="15" t="s">
+      <c r="R110" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S110" s="16" t="s">
         <v>786</v>
       </c>
-      <c r="T110" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U110" s="15">
+      <c r="T110" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U110" s="16">
         <v>85.0</v>
       </c>
-      <c r="V110" s="15">
+      <c r="V110" s="16">
         <v>0.0</v>
       </c>
-      <c r="W110" s="15">
+      <c r="W110" s="16">
         <v>3088.0</v>
       </c>
-      <c r="X110" s="15">
+      <c r="X110" s="16">
         <v>892.0</v>
       </c>
-      <c r="Y110" s="15">
+      <c r="Y110" s="16">
         <v>17806.0</v>
       </c>
-      <c r="Z110" s="15">
+      <c r="Z110" s="16">
         <v>623.0</v>
       </c>
-      <c r="AA110" s="15">
+      <c r="AA110" s="16">
         <v>19474.0</v>
       </c>
-      <c r="AB110" s="15">
+      <c r="AB110" s="16">
         <v>15.0</v>
       </c>
-      <c r="AC110" s="15">
+      <c r="AC110" s="16">
         <v>2164.0</v>
       </c>
-      <c r="AD110" s="15">
+      <c r="AD110" s="16">
         <v>1523880.0</v>
       </c>
-      <c r="AE110" s="18">
+      <c r="AE110" s="19">
         <v>46239.0</v>
       </c>
-      <c r="AF110" s="15">
+      <c r="AF110" s="16">
         <v>53.0</v>
       </c>
-      <c r="AG110" s="15" t="s">
+      <c r="AG110" s="16" t="s">
         <v>784</v>
       </c>
-      <c r="AH110" s="19" t="s">
+      <c r="AH110" s="20" t="s">
         <v>785</v>
       </c>
-      <c r="AI110" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ110" s="15" t="s">
+      <c r="AI110" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ110" s="16" t="s">
         <v>786</v>
       </c>
-      <c r="AK110" s="19" t="s">
+      <c r="AK110" s="20" t="s">
         <v>787</v>
       </c>
-      <c r="AL110" s="20"/>
-      <c r="AM110" s="20"/>
-      <c r="AN110" s="20"/>
-      <c r="AO110" s="20"/>
-      <c r="AP110" s="20"/>
-      <c r="AQ110" s="20"/>
-      <c r="AR110" s="20"/>
-      <c r="AS110" s="20"/>
-      <c r="AT110" s="20"/>
-      <c r="AU110" s="20"/>
-      <c r="AV110" s="21"/>
-      <c r="AW110" s="21"/>
-      <c r="AX110" s="21"/>
-      <c r="AY110" s="21"/>
-      <c r="AZ110" s="21"/>
-      <c r="BA110" s="21"/>
-      <c r="BB110" s="21"/>
-      <c r="BC110" s="21"/>
-      <c r="BD110" s="21"/>
+      <c r="AL110" s="21"/>
+      <c r="AM110" s="21"/>
+      <c r="AN110" s="21"/>
+      <c r="AO110" s="21"/>
+      <c r="AP110" s="21"/>
+      <c r="AQ110" s="21"/>
+      <c r="AR110" s="21"/>
+      <c r="AS110" s="21"/>
+      <c r="AT110" s="21"/>
+      <c r="AU110" s="21"/>
+      <c r="AV110" s="22"/>
+      <c r="AW110" s="22"/>
+      <c r="AX110" s="22"/>
+      <c r="AY110" s="22"/>
+      <c r="AZ110" s="22"/>
+      <c r="BA110" s="22"/>
+      <c r="BB110" s="22"/>
+      <c r="BC110" s="22"/>
+      <c r="BD110" s="22"/>
     </row>
     <row r="111">
-      <c r="A111" s="15">
+      <c r="A111" s="16">
         <v>35.0</v>
       </c>
-      <c r="B111" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C111" s="15" t="s">
+      <c r="B111" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C111" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D111" s="16">
+      <c r="D111" s="17">
         <v>46174.71189814815</v>
       </c>
-      <c r="E111" s="15">
+      <c r="E111" s="16">
         <v>4.29315541090758E15</v>
       </c>
-      <c r="F111" s="15" t="b">
+      <c r="F111" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G111" s="15" t="s">
+      <c r="G111" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H111" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I111" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J111" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K111" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L111" s="15" t="s">
+      <c r="H111" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I111" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J111" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K111" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L111" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M111" s="17" t="s">
+      <c r="M111" s="18" t="s">
         <v>788</v>
       </c>
-      <c r="N111" s="16">
+      <c r="N111" s="17">
         <v>46174.72278935185</v>
       </c>
-      <c r="O111" s="15" t="s">
+      <c r="O111" s="16" t="s">
         <v>789</v>
       </c>
-      <c r="P111" s="15" t="s">
+      <c r="P111" s="16" t="s">
         <v>790</v>
       </c>
-      <c r="Q111" s="15" t="s">
+      <c r="Q111" s="16" t="s">
         <v>791</v>
       </c>
-      <c r="R111" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S111" s="17" t="s">
+      <c r="R111" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S111" s="18" t="s">
         <v>792</v>
       </c>
-      <c r="T111" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U111" s="15">
+      <c r="T111" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U111" s="16">
         <v>304.0</v>
       </c>
-      <c r="V111" s="15">
+      <c r="V111" s="16">
         <v>0.0</v>
       </c>
-      <c r="W111" s="15">
+      <c r="W111" s="16">
         <v>3949.0</v>
       </c>
-      <c r="X111" s="15">
+      <c r="X111" s="16">
         <v>937.0</v>
       </c>
-      <c r="Y111" s="15">
+      <c r="Y111" s="16">
         <v>16246.0</v>
       </c>
-      <c r="Z111" s="15">
+      <c r="Z111" s="16">
         <v>855.0</v>
       </c>
-      <c r="AA111" s="15">
+      <c r="AA111" s="16">
         <v>18376.0</v>
       </c>
-      <c r="AB111" s="15">
+      <c r="AB111" s="16">
         <v>8.0</v>
       </c>
-      <c r="AC111" s="15">
+      <c r="AC111" s="16">
         <v>3623.0</v>
       </c>
-      <c r="AD111" s="15">
+      <c r="AD111" s="16">
         <v>626262.0</v>
       </c>
-      <c r="AE111" s="18">
+      <c r="AE111" s="19">
         <v>46239.0</v>
       </c>
-      <c r="AF111" s="15">
+      <c r="AF111" s="16">
         <v>26.0</v>
       </c>
-      <c r="AG111" s="15" t="s">
+      <c r="AG111" s="16" t="s">
         <v>790</v>
       </c>
-      <c r="AH111" s="19" t="s">
+      <c r="AH111" s="20" t="s">
         <v>791</v>
       </c>
-      <c r="AI111" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ111" s="17" t="s">
+      <c r="AI111" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ111" s="18" t="s">
         <v>792</v>
       </c>
-      <c r="AK111" s="19" t="s">
+      <c r="AK111" s="20" t="s">
         <v>793</v>
       </c>
-      <c r="AL111" s="20"/>
-      <c r="AM111" s="20"/>
-      <c r="AN111" s="20"/>
-      <c r="AO111" s="20"/>
-      <c r="AP111" s="20"/>
-      <c r="AQ111" s="20"/>
-      <c r="AR111" s="20"/>
-      <c r="AS111" s="20"/>
-      <c r="AT111" s="20"/>
-      <c r="AU111" s="20"/>
-      <c r="AV111" s="21"/>
-      <c r="AW111" s="21"/>
-      <c r="AX111" s="21"/>
-      <c r="AY111" s="21"/>
-      <c r="AZ111" s="21"/>
-      <c r="BA111" s="21"/>
-      <c r="BB111" s="21"/>
-      <c r="BC111" s="21"/>
-      <c r="BD111" s="21"/>
+      <c r="AL111" s="21"/>
+      <c r="AM111" s="21"/>
+      <c r="AN111" s="21"/>
+      <c r="AO111" s="21"/>
+      <c r="AP111" s="21"/>
+      <c r="AQ111" s="21"/>
+      <c r="AR111" s="21"/>
+      <c r="AS111" s="21"/>
+      <c r="AT111" s="21"/>
+      <c r="AU111" s="21"/>
+      <c r="AV111" s="22"/>
+      <c r="AW111" s="22"/>
+      <c r="AX111" s="22"/>
+      <c r="AY111" s="22"/>
+      <c r="AZ111" s="22"/>
+      <c r="BA111" s="22"/>
+      <c r="BB111" s="22"/>
+      <c r="BC111" s="22"/>
+      <c r="BD111" s="22"/>
     </row>
     <row r="112">
-      <c r="A112" s="15">
+      <c r="A112" s="16">
         <v>36.0</v>
       </c>
-      <c r="B112" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C112" s="15" t="s">
+      <c r="B112" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C112" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D112" s="16">
+      <c r="D112" s="17">
         <v>46174.85824074074</v>
       </c>
-      <c r="E112" s="15">
+      <c r="E112" s="16">
         <v>1.55809310917362E15</v>
       </c>
-      <c r="F112" s="15" t="b">
+      <c r="F112" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G112" s="15" t="s">
+      <c r="G112" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H112" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I112" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J112" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K112" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L112" s="15" t="s">
+      <c r="H112" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I112" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J112" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K112" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L112" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M112" s="17" t="s">
+      <c r="M112" s="18" t="s">
         <v>794</v>
       </c>
-      <c r="N112" s="16">
+      <c r="N112" s="17">
         <v>46178.01967592593</v>
       </c>
-      <c r="O112" s="15" t="s">
+      <c r="O112" s="16" t="s">
         <v>795</v>
       </c>
-      <c r="P112" s="15">
+      <c r="P112" s="16">
         <v>9.55382885966988E14</v>
       </c>
-      <c r="Q112" s="17" t="s">
+      <c r="Q112" s="18" t="s">
         <v>796</v>
       </c>
-      <c r="R112" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S112" s="15" t="s">
+      <c r="R112" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S112" s="16" t="s">
         <v>797</v>
       </c>
-      <c r="T112" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U112" s="15">
+      <c r="T112" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U112" s="16">
         <v>395.0</v>
       </c>
-      <c r="V112" s="15">
+      <c r="V112" s="16">
         <v>0.0</v>
       </c>
-      <c r="W112" s="15">
+      <c r="W112" s="16">
         <v>6443.0</v>
       </c>
-      <c r="X112" s="15">
+      <c r="X112" s="16">
         <v>1101.0</v>
       </c>
-      <c r="Y112" s="15">
+      <c r="Y112" s="16">
         <v>15291.0</v>
       </c>
-      <c r="Z112" s="15">
+      <c r="Z112" s="16">
         <v>202.0</v>
       </c>
-      <c r="AA112" s="15">
+      <c r="AA112" s="16">
         <v>17954.0</v>
       </c>
-      <c r="AB112" s="15">
+      <c r="AB112" s="16">
         <v>26.0</v>
       </c>
-      <c r="AC112" s="15">
+      <c r="AC112" s="16">
         <v>24198.0</v>
       </c>
-      <c r="AD112" s="15">
+      <c r="AD112" s="16">
         <v>830554.0</v>
       </c>
-      <c r="AE112" s="18">
+      <c r="AE112" s="19">
         <v>46241.0</v>
       </c>
-      <c r="AF112" s="15">
+      <c r="AF112" s="16">
         <v>939.0</v>
       </c>
-      <c r="AG112" s="15">
+      <c r="AG112" s="16">
         <v>9.55382885966988E14</v>
       </c>
-      <c r="AH112" s="22" t="s">
+      <c r="AH112" s="23" t="s">
         <v>796</v>
       </c>
-      <c r="AI112" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ112" s="15" t="s">
+      <c r="AI112" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ112" s="16" t="s">
         <v>797</v>
       </c>
-      <c r="AK112" s="19" t="s">
+      <c r="AK112" s="20" t="s">
         <v>798</v>
       </c>
-      <c r="AL112" s="20"/>
-      <c r="AM112" s="20"/>
-      <c r="AN112" s="20"/>
-      <c r="AO112" s="20"/>
-      <c r="AP112" s="20"/>
-      <c r="AQ112" s="20"/>
-      <c r="AR112" s="20"/>
-      <c r="AS112" s="20"/>
-      <c r="AT112" s="20"/>
-      <c r="AU112" s="20"/>
-      <c r="AV112" s="21"/>
-      <c r="AW112" s="21"/>
-      <c r="AX112" s="21"/>
-      <c r="AY112" s="21"/>
-      <c r="AZ112" s="21"/>
-      <c r="BA112" s="21"/>
-      <c r="BB112" s="21"/>
-      <c r="BC112" s="21"/>
-      <c r="BD112" s="21"/>
+      <c r="AL112" s="21"/>
+      <c r="AM112" s="21"/>
+      <c r="AN112" s="21"/>
+      <c r="AO112" s="21"/>
+      <c r="AP112" s="21"/>
+      <c r="AQ112" s="21"/>
+      <c r="AR112" s="21"/>
+      <c r="AS112" s="21"/>
+      <c r="AT112" s="21"/>
+      <c r="AU112" s="21"/>
+      <c r="AV112" s="22"/>
+      <c r="AW112" s="22"/>
+      <c r="AX112" s="22"/>
+      <c r="AY112" s="22"/>
+      <c r="AZ112" s="22"/>
+      <c r="BA112" s="22"/>
+      <c r="BB112" s="22"/>
+      <c r="BC112" s="22"/>
+      <c r="BD112" s="22"/>
     </row>
     <row r="113">
-      <c r="A113" s="15">
+      <c r="A113" s="16">
         <v>45.0</v>
       </c>
-      <c r="B113" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C113" s="15" t="s">
+      <c r="B113" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C113" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="D113" s="16">
+      <c r="D113" s="17">
         <v>46173.501493055555</v>
       </c>
-      <c r="E113" s="15" t="s">
+      <c r="E113" s="16" t="s">
         <v>799</v>
       </c>
-      <c r="F113" s="15" t="b">
+      <c r="F113" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G113" s="15" t="s">
+      <c r="G113" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H113" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I113" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J113" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K113" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L113" s="15" t="s">
+      <c r="H113" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I113" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J113" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K113" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L113" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M113" s="17" t="s">
+      <c r="M113" s="18" t="s">
         <v>800</v>
       </c>
-      <c r="N113" s="16">
+      <c r="N113" s="17">
         <v>46173.505902777775</v>
       </c>
-      <c r="O113" s="15" t="s">
+      <c r="O113" s="16" t="s">
         <v>801</v>
       </c>
-      <c r="P113" s="15">
+      <c r="P113" s="16">
         <v>7.36914604690384E14</v>
       </c>
-      <c r="Q113" s="15" t="s">
+      <c r="Q113" s="16" t="s">
         <v>802</v>
       </c>
-      <c r="R113" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S113" s="15" t="s">
+      <c r="R113" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S113" s="16" t="s">
         <v>803</v>
       </c>
-      <c r="T113" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U113" s="15">
+      <c r="T113" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U113" s="16">
         <v>598.0</v>
       </c>
-      <c r="V113" s="15">
+      <c r="V113" s="16">
         <v>0.0</v>
       </c>
-      <c r="W113" s="15">
+      <c r="W113" s="16">
         <v>5404.0</v>
       </c>
-      <c r="X113" s="15">
+      <c r="X113" s="16">
         <v>1450.0</v>
       </c>
-      <c r="Y113" s="15">
+      <c r="Y113" s="16">
         <v>11583.0</v>
       </c>
-      <c r="Z113" s="15">
+      <c r="Z113" s="16">
         <v>1920.0</v>
       </c>
-      <c r="AA113" s="15">
+      <c r="AA113" s="16">
         <v>15596.0</v>
       </c>
-      <c r="AB113" s="15">
+      <c r="AB113" s="16">
         <v>21.0</v>
       </c>
-      <c r="AC113" s="15">
+      <c r="AC113" s="16">
         <v>649.0</v>
       </c>
-      <c r="AD113" s="15">
+      <c r="AD113" s="16">
         <v>434964.0</v>
       </c>
-      <c r="AE113" s="18">
+      <c r="AE113" s="19">
         <v>46239.0</v>
       </c>
-      <c r="AF113" s="15">
+      <c r="AF113" s="16">
         <v>24.0</v>
       </c>
-      <c r="AG113" s="15">
+      <c r="AG113" s="16">
         <v>7.36914604690384E14</v>
       </c>
-      <c r="AH113" s="19" t="s">
+      <c r="AH113" s="20" t="s">
         <v>802</v>
       </c>
-      <c r="AI113" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ113" s="15" t="s">
+      <c r="AI113" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ113" s="16" t="s">
         <v>803</v>
       </c>
-      <c r="AK113" s="19" t="s">
+      <c r="AK113" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="AL113" s="20"/>
-      <c r="AM113" s="20"/>
-      <c r="AN113" s="20"/>
-      <c r="AO113" s="20"/>
-      <c r="AP113" s="20"/>
-      <c r="AQ113" s="20"/>
-      <c r="AR113" s="20"/>
-      <c r="AS113" s="20"/>
-      <c r="AT113" s="20"/>
-      <c r="AU113" s="20"/>
-      <c r="AV113" s="21"/>
-      <c r="AW113" s="21"/>
-      <c r="AX113" s="21"/>
-      <c r="AY113" s="21"/>
-      <c r="AZ113" s="21"/>
-      <c r="BA113" s="21"/>
-      <c r="BB113" s="21"/>
-      <c r="BC113" s="21"/>
-      <c r="BD113" s="21"/>
+      <c r="AL113" s="21"/>
+      <c r="AM113" s="21"/>
+      <c r="AN113" s="21"/>
+      <c r="AO113" s="21"/>
+      <c r="AP113" s="21"/>
+      <c r="AQ113" s="21"/>
+      <c r="AR113" s="21"/>
+      <c r="AS113" s="21"/>
+      <c r="AT113" s="21"/>
+      <c r="AU113" s="21"/>
+      <c r="AV113" s="22"/>
+      <c r="AW113" s="22"/>
+      <c r="AX113" s="22"/>
+      <c r="AY113" s="22"/>
+      <c r="AZ113" s="22"/>
+      <c r="BA113" s="22"/>
+      <c r="BB113" s="22"/>
+      <c r="BC113" s="22"/>
+      <c r="BD113" s="22"/>
     </row>
     <row r="114">
-      <c r="A114" s="15">
+      <c r="A114" s="16">
         <v>48.0</v>
       </c>
-      <c r="B114" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C114" s="15" t="s">
+      <c r="B114" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C114" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D114" s="16">
+      <c r="D114" s="17">
         <v>46174.07329861111</v>
       </c>
-      <c r="E114" s="15" t="s">
+      <c r="E114" s="16" t="s">
         <v>805</v>
       </c>
-      <c r="F114" s="15" t="b">
+      <c r="F114" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G114" s="15" t="s">
+      <c r="G114" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H114" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I114" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J114" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K114" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L114" s="15" t="s">
+      <c r="H114" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I114" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J114" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K114" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L114" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M114" s="17" t="s">
+      <c r="M114" s="18" t="s">
         <v>806</v>
       </c>
-      <c r="N114" s="16">
+      <c r="N114" s="17">
         <v>46174.08373842593</v>
       </c>
-      <c r="O114" s="15" t="s">
+      <c r="O114" s="16" t="s">
         <v>807</v>
       </c>
-      <c r="P114" s="15" t="s">
+      <c r="P114" s="16" t="s">
         <v>784</v>
       </c>
-      <c r="Q114" s="15" t="s">
+      <c r="Q114" s="16" t="s">
         <v>785</v>
       </c>
-      <c r="R114" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S114" s="15" t="s">
+      <c r="R114" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S114" s="16" t="s">
         <v>786</v>
       </c>
-      <c r="T114" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U114" s="15">
+      <c r="T114" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U114" s="16">
         <v>31.0</v>
       </c>
-      <c r="V114" s="15">
+      <c r="V114" s="16">
         <v>0.0</v>
       </c>
-      <c r="W114" s="15">
+      <c r="W114" s="16">
         <v>1462.0</v>
       </c>
-      <c r="X114" s="15">
+      <c r="X114" s="16">
         <v>608.0</v>
       </c>
-      <c r="Y114" s="15">
+      <c r="Y114" s="16">
         <v>13216.0</v>
       </c>
-      <c r="Z114" s="15">
+      <c r="Z114" s="16">
         <v>426.0</v>
       </c>
-      <c r="AA114" s="15">
+      <c r="AA114" s="16">
         <v>14349.0</v>
       </c>
-      <c r="AB114" s="15">
+      <c r="AB114" s="16">
         <v>36.0</v>
       </c>
-      <c r="AC114" s="15">
+      <c r="AC114" s="16">
         <v>1227.0</v>
       </c>
-      <c r="AD114" s="15">
+      <c r="AD114" s="16">
         <v>568044.0</v>
       </c>
-      <c r="AE114" s="18">
+      <c r="AE114" s="19">
         <v>46239.0</v>
       </c>
-      <c r="AF114" s="15">
+      <c r="AF114" s="16">
         <v>32.0</v>
       </c>
-      <c r="AG114" s="15" t="s">
+      <c r="AG114" s="16" t="s">
         <v>784</v>
       </c>
-      <c r="AH114" s="19" t="s">
+      <c r="AH114" s="20" t="s">
         <v>785</v>
       </c>
-      <c r="AI114" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ114" s="15" t="s">
+      <c r="AI114" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ114" s="16" t="s">
         <v>786</v>
       </c>
-      <c r="AK114" s="19" t="s">
+      <c r="AK114" s="20" t="s">
         <v>808</v>
       </c>
-      <c r="AL114" s="20"/>
-      <c r="AM114" s="20"/>
-      <c r="AN114" s="20"/>
-      <c r="AO114" s="20"/>
-      <c r="AP114" s="20"/>
-      <c r="AQ114" s="20"/>
-      <c r="AR114" s="20"/>
-      <c r="AS114" s="20"/>
-      <c r="AT114" s="20"/>
-      <c r="AU114" s="20"/>
-      <c r="AV114" s="21"/>
-      <c r="AW114" s="21"/>
-      <c r="AX114" s="21"/>
-      <c r="AY114" s="21"/>
-      <c r="AZ114" s="21"/>
-      <c r="BA114" s="21"/>
-      <c r="BB114" s="21"/>
-      <c r="BC114" s="21"/>
-      <c r="BD114" s="21"/>
+      <c r="AL114" s="21"/>
+      <c r="AM114" s="21"/>
+      <c r="AN114" s="21"/>
+      <c r="AO114" s="21"/>
+      <c r="AP114" s="21"/>
+      <c r="AQ114" s="21"/>
+      <c r="AR114" s="21"/>
+      <c r="AS114" s="21"/>
+      <c r="AT114" s="21"/>
+      <c r="AU114" s="21"/>
+      <c r="AV114" s="22"/>
+      <c r="AW114" s="22"/>
+      <c r="AX114" s="22"/>
+      <c r="AY114" s="22"/>
+      <c r="AZ114" s="22"/>
+      <c r="BA114" s="22"/>
+      <c r="BB114" s="22"/>
+      <c r="BC114" s="22"/>
+      <c r="BD114" s="22"/>
     </row>
     <row r="115">
-      <c r="A115" s="15">
+      <c r="A115" s="16">
         <v>53.0</v>
       </c>
-      <c r="B115" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C115" s="15" t="s">
+      <c r="B115" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C115" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D115" s="16">
+      <c r="D115" s="17">
         <v>46173.81659722222</v>
       </c>
-      <c r="E115" s="15" t="s">
+      <c r="E115" s="16" t="s">
         <v>809</v>
       </c>
-      <c r="F115" s="15" t="b">
+      <c r="F115" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G115" s="15" t="s">
+      <c r="G115" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H115" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I115" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J115" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K115" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L115" s="15" t="s">
+      <c r="H115" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I115" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J115" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K115" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L115" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M115" s="17" t="s">
+      <c r="M115" s="18" t="s">
         <v>810</v>
       </c>
-      <c r="N115" s="16">
+      <c r="N115" s="17">
         <v>46173.83131944444</v>
       </c>
-      <c r="O115" s="15" t="s">
+      <c r="O115" s="16" t="s">
         <v>811</v>
       </c>
-      <c r="P115" s="15" t="s">
+      <c r="P115" s="16" t="s">
         <v>812</v>
       </c>
-      <c r="Q115" s="15" t="s">
+      <c r="Q115" s="16" t="s">
         <v>813</v>
       </c>
-      <c r="R115" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S115" s="17" t="s">
+      <c r="R115" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S115" s="18" t="s">
         <v>814</v>
       </c>
-      <c r="T115" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U115" s="15">
+      <c r="T115" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U115" s="16">
         <v>23.0</v>
       </c>
-      <c r="V115" s="15">
+      <c r="V115" s="16">
         <v>0.0</v>
       </c>
-      <c r="W115" s="15">
+      <c r="W115" s="16">
         <v>507.0</v>
       </c>
-      <c r="X115" s="15">
+      <c r="X115" s="16">
         <v>1576.0</v>
       </c>
-      <c r="Y115" s="15">
+      <c r="Y115" s="16">
         <v>9856.0</v>
       </c>
-      <c r="Z115" s="15">
+      <c r="Z115" s="16">
         <v>1463.0</v>
       </c>
-      <c r="AA115" s="15">
+      <c r="AA115" s="16">
         <v>12933.0</v>
       </c>
-      <c r="AB115" s="15">
+      <c r="AB115" s="16">
         <v>4.0</v>
       </c>
-      <c r="AC115" s="15">
+      <c r="AC115" s="16">
         <v>952.0</v>
       </c>
-      <c r="AD115" s="15">
+      <c r="AD115" s="16">
         <v>546475.0</v>
       </c>
-      <c r="AE115" s="18">
+      <c r="AE115" s="19">
         <v>46239.0</v>
       </c>
-      <c r="AF115" s="15">
+      <c r="AF115" s="16">
         <v>11.0</v>
       </c>
-      <c r="AG115" s="15" t="s">
+      <c r="AG115" s="16" t="s">
         <v>812</v>
       </c>
-      <c r="AH115" s="19" t="s">
+      <c r="AH115" s="20" t="s">
         <v>813</v>
       </c>
-      <c r="AI115" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ115" s="17" t="s">
+      <c r="AI115" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ115" s="18" t="s">
         <v>814</v>
       </c>
-      <c r="AK115" s="19" t="s">
+      <c r="AK115" s="20" t="s">
         <v>815</v>
       </c>
-      <c r="AL115" s="20"/>
-      <c r="AM115" s="20"/>
-      <c r="AN115" s="20"/>
-      <c r="AO115" s="20"/>
-      <c r="AP115" s="20"/>
-      <c r="AQ115" s="20"/>
-      <c r="AR115" s="20"/>
-      <c r="AS115" s="20"/>
-      <c r="AT115" s="20"/>
-      <c r="AU115" s="20"/>
-      <c r="AV115" s="21"/>
-      <c r="AW115" s="21"/>
-      <c r="AX115" s="21"/>
-      <c r="AY115" s="21"/>
-      <c r="AZ115" s="21"/>
-      <c r="BA115" s="21"/>
-      <c r="BB115" s="21"/>
-      <c r="BC115" s="21"/>
-      <c r="BD115" s="21"/>
+      <c r="AL115" s="21"/>
+      <c r="AM115" s="21"/>
+      <c r="AN115" s="21"/>
+      <c r="AO115" s="21"/>
+      <c r="AP115" s="21"/>
+      <c r="AQ115" s="21"/>
+      <c r="AR115" s="21"/>
+      <c r="AS115" s="21"/>
+      <c r="AT115" s="21"/>
+      <c r="AU115" s="21"/>
+      <c r="AV115" s="22"/>
+      <c r="AW115" s="22"/>
+      <c r="AX115" s="22"/>
+      <c r="AY115" s="22"/>
+      <c r="AZ115" s="22"/>
+      <c r="BA115" s="22"/>
+      <c r="BB115" s="22"/>
+      <c r="BC115" s="22"/>
+      <c r="BD115" s="22"/>
     </row>
     <row r="116">
-      <c r="A116" s="15">
+      <c r="A116" s="16">
         <v>79.0</v>
       </c>
-      <c r="B116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C116" s="15" t="s">
+      <c r="B116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C116" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D116" s="16">
+      <c r="D116" s="17">
         <v>46173.52134259259</v>
       </c>
-      <c r="E116" s="15" t="s">
+      <c r="E116" s="16" t="s">
         <v>816</v>
       </c>
-      <c r="F116" s="15" t="b">
+      <c r="F116" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G116" s="15" t="s">
+      <c r="G116" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L116" s="15" t="s">
+      <c r="H116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L116" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M116" s="17" t="s">
+      <c r="M116" s="18" t="s">
         <v>817</v>
       </c>
-      <c r="N116" s="16">
+      <c r="N116" s="17">
         <v>46173.56346064815</v>
       </c>
-      <c r="O116" s="15" t="s">
+      <c r="O116" s="16" t="s">
         <v>818</v>
       </c>
-      <c r="P116" s="15" t="s">
+      <c r="P116" s="16" t="s">
         <v>819</v>
       </c>
-      <c r="Q116" s="15" t="s">
+      <c r="Q116" s="16" t="s">
         <v>820</v>
       </c>
-      <c r="R116" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="T116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U116" s="15">
+      <c r="R116" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="T116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U116" s="16">
         <v>4.0</v>
       </c>
-      <c r="V116" s="15">
+      <c r="V116" s="16">
         <v>0.0</v>
       </c>
-      <c r="W116" s="15">
+      <c r="W116" s="16">
         <v>1440.0</v>
       </c>
-      <c r="X116" s="15">
+      <c r="X116" s="16">
         <v>35.0</v>
       </c>
-      <c r="Y116" s="15">
+      <c r="Y116" s="16">
         <v>8419.0</v>
       </c>
-      <c r="Z116" s="15">
+      <c r="Z116" s="16">
         <v>538.0</v>
       </c>
-      <c r="AA116" s="15">
+      <c r="AA116" s="16">
         <v>9001.0</v>
       </c>
-      <c r="AB116" s="15">
+      <c r="AB116" s="16">
         <v>3.0</v>
       </c>
-      <c r="AC116" s="15">
+      <c r="AC116" s="16">
         <v>1134.0</v>
       </c>
-      <c r="AD116" s="15">
+      <c r="AD116" s="16">
         <v>95985.0</v>
       </c>
-      <c r="AE116" s="18">
+      <c r="AE116" s="19">
         <v>46239.0</v>
       </c>
-      <c r="AF116" s="15">
+      <c r="AF116" s="16">
         <v>2.0</v>
       </c>
-      <c r="AG116" s="15" t="s">
+      <c r="AG116" s="16" t="s">
         <v>819</v>
       </c>
-      <c r="AH116" s="19" t="s">
+      <c r="AH116" s="20" t="s">
         <v>820</v>
       </c>
-      <c r="AI116" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ116" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="AK116" s="19" t="s">
+      <c r="AI116" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ116" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK116" s="20" t="s">
         <v>821</v>
       </c>
-      <c r="AL116" s="20"/>
-      <c r="AM116" s="20"/>
-      <c r="AN116" s="20"/>
-      <c r="AO116" s="20"/>
-      <c r="AP116" s="20"/>
-      <c r="AQ116" s="20"/>
-      <c r="AR116" s="20"/>
-      <c r="AS116" s="20"/>
-      <c r="AT116" s="20"/>
-      <c r="AU116" s="20"/>
-      <c r="AV116" s="21"/>
-      <c r="AW116" s="21"/>
-      <c r="AX116" s="21"/>
-      <c r="AY116" s="21"/>
-      <c r="AZ116" s="21"/>
-      <c r="BA116" s="21"/>
-      <c r="BB116" s="21"/>
-      <c r="BC116" s="21"/>
-      <c r="BD116" s="21"/>
+      <c r="AL116" s="21"/>
+      <c r="AM116" s="21"/>
+      <c r="AN116" s="21"/>
+      <c r="AO116" s="21"/>
+      <c r="AP116" s="21"/>
+      <c r="AQ116" s="21"/>
+      <c r="AR116" s="21"/>
+      <c r="AS116" s="21"/>
+      <c r="AT116" s="21"/>
+      <c r="AU116" s="21"/>
+      <c r="AV116" s="22"/>
+      <c r="AW116" s="22"/>
+      <c r="AX116" s="22"/>
+      <c r="AY116" s="22"/>
+      <c r="AZ116" s="22"/>
+      <c r="BA116" s="22"/>
+      <c r="BB116" s="22"/>
+      <c r="BC116" s="22"/>
+      <c r="BD116" s="22"/>
     </row>
     <row r="117">
-      <c r="A117" s="15">
+      <c r="A117" s="16">
         <v>84.0</v>
       </c>
-      <c r="B117" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C117" s="15" t="s">
+      <c r="B117" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C117" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="D117" s="16">
+      <c r="D117" s="17">
         <v>46173.92109953704</v>
       </c>
-      <c r="E117" s="15" t="s">
+      <c r="E117" s="16" t="s">
         <v>822</v>
       </c>
-      <c r="F117" s="15" t="b">
+      <c r="F117" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G117" s="15" t="s">
+      <c r="G117" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H117" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I117" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J117" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K117" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L117" s="15" t="s">
+      <c r="H117" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I117" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J117" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K117" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L117" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M117" s="17" t="s">
+      <c r="M117" s="18" t="s">
         <v>823</v>
       </c>
-      <c r="N117" s="16">
+      <c r="N117" s="17">
         <v>46173.92493055556</v>
       </c>
-      <c r="O117" s="15" t="s">
+      <c r="O117" s="16" t="s">
         <v>824</v>
       </c>
-      <c r="P117" s="15">
+      <c r="P117" s="16">
         <v>1.87342180404848E15</v>
       </c>
-      <c r="Q117" s="15" t="s">
+      <c r="Q117" s="16" t="s">
         <v>825</v>
       </c>
-      <c r="R117" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S117" s="15" t="s">
+      <c r="R117" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S117" s="16" t="s">
         <v>826</v>
       </c>
-      <c r="T117" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U117" s="15">
+      <c r="T117" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U117" s="16">
         <v>1743.0</v>
       </c>
-      <c r="V117" s="15">
+      <c r="V117" s="16">
         <v>0.0</v>
       </c>
-      <c r="W117" s="15">
+      <c r="W117" s="16">
         <v>2716.0</v>
       </c>
-      <c r="X117" s="15">
+      <c r="X117" s="16">
         <v>164.0</v>
       </c>
-      <c r="Y117" s="15">
+      <c r="Y117" s="16">
         <v>1750.0</v>
       </c>
-      <c r="Z117" s="15">
+      <c r="Z117" s="16">
         <v>349.0</v>
       </c>
-      <c r="AA117" s="15">
+      <c r="AA117" s="16">
         <v>8401.0</v>
       </c>
-      <c r="AB117" s="15">
+      <c r="AB117" s="16">
         <v>4333.0</v>
       </c>
-      <c r="AC117" s="15">
+      <c r="AC117" s="16">
         <v>264.0</v>
       </c>
-      <c r="AD117" s="15">
+      <c r="AD117" s="16">
         <v>401236.0</v>
       </c>
-      <c r="AE117" s="18">
+      <c r="AE117" s="19">
         <v>46239.0</v>
       </c>
-      <c r="AF117" s="15">
+      <c r="AF117" s="16">
         <v>62.0</v>
       </c>
-      <c r="AG117" s="15">
+      <c r="AG117" s="16">
         <v>1.87342180404848E15</v>
       </c>
-      <c r="AH117" s="19" t="s">
+      <c r="AH117" s="20" t="s">
         <v>825</v>
       </c>
-      <c r="AI117" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ117" s="15" t="s">
+      <c r="AI117" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ117" s="16" t="s">
         <v>826</v>
       </c>
-      <c r="AK117" s="19" t="s">
+      <c r="AK117" s="20" t="s">
         <v>827</v>
       </c>
-      <c r="AL117" s="23"/>
-      <c r="AM117" s="23"/>
-      <c r="AN117" s="23"/>
-      <c r="AO117" s="23"/>
-      <c r="AP117" s="23"/>
-      <c r="AQ117" s="23"/>
-      <c r="AR117" s="23"/>
-      <c r="AS117" s="23"/>
-      <c r="AT117" s="23"/>
-      <c r="AU117" s="23"/>
-      <c r="AV117" s="19"/>
-      <c r="AW117" s="19"/>
-      <c r="AX117" s="19"/>
-      <c r="AY117" s="19"/>
-      <c r="AZ117" s="19"/>
-      <c r="BA117" s="21"/>
-      <c r="BB117" s="19"/>
-      <c r="BC117" s="19"/>
-      <c r="BD117" s="21"/>
+      <c r="AL117" s="24"/>
+      <c r="AM117" s="24"/>
+      <c r="AN117" s="24"/>
+      <c r="AO117" s="24"/>
+      <c r="AP117" s="24"/>
+      <c r="AQ117" s="24"/>
+      <c r="AR117" s="24"/>
+      <c r="AS117" s="24"/>
+      <c r="AT117" s="24"/>
+      <c r="AU117" s="24"/>
+      <c r="AV117" s="20"/>
+      <c r="AW117" s="20"/>
+      <c r="AX117" s="20"/>
+      <c r="AY117" s="20"/>
+      <c r="AZ117" s="20"/>
+      <c r="BA117" s="22"/>
+      <c r="BB117" s="20"/>
+      <c r="BC117" s="20"/>
+      <c r="BD117" s="22"/>
     </row>
     <row r="118">
-      <c r="A118" s="15">
+      <c r="A118" s="16">
         <v>85.0</v>
       </c>
-      <c r="B118" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C118" s="15" t="s">
+      <c r="B118" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C118" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D118" s="16">
+      <c r="D118" s="17">
         <v>46173.7622337963</v>
       </c>
-      <c r="E118" s="15" t="s">
+      <c r="E118" s="16" t="s">
         <v>828</v>
       </c>
-      <c r="F118" s="15" t="b">
+      <c r="F118" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G118" s="15" t="s">
+      <c r="G118" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H118" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I118" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J118" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K118" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L118" s="15" t="s">
+      <c r="H118" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I118" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J118" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K118" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L118" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M118" s="17" t="s">
+      <c r="M118" s="18" t="s">
         <v>829</v>
       </c>
-      <c r="N118" s="16">
+      <c r="N118" s="17">
         <v>46174.59012731481</v>
       </c>
-      <c r="O118" s="15" t="s">
+      <c r="O118" s="16" t="s">
         <v>830</v>
       </c>
-      <c r="P118" s="15" t="s">
+      <c r="P118" s="16" t="s">
         <v>831</v>
       </c>
-      <c r="Q118" s="15" t="s">
+      <c r="Q118" s="16" t="s">
         <v>832</v>
       </c>
-      <c r="R118" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S118" s="15" t="s">
+      <c r="R118" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S118" s="16" t="s">
         <v>833</v>
       </c>
-      <c r="T118" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U118" s="15">
+      <c r="T118" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U118" s="16">
         <v>2.0</v>
       </c>
-      <c r="V118" s="15">
+      <c r="V118" s="16">
         <v>0.0</v>
       </c>
-      <c r="W118" s="15">
+      <c r="W118" s="16">
         <v>118.0</v>
       </c>
-      <c r="X118" s="15">
+      <c r="X118" s="16">
         <v>1908.0</v>
       </c>
-      <c r="Y118" s="15">
+      <c r="Y118" s="16">
         <v>5893.0</v>
       </c>
-      <c r="Z118" s="15">
+      <c r="Z118" s="16">
         <v>91.0</v>
       </c>
-      <c r="AA118" s="15">
+      <c r="AA118" s="16">
         <v>7900.0</v>
       </c>
-      <c r="AB118" s="15">
+      <c r="AB118" s="16">
         <v>2.0</v>
       </c>
-      <c r="AC118" s="15">
+      <c r="AC118" s="16">
         <v>752.0</v>
       </c>
-      <c r="AD118" s="15">
+      <c r="AD118" s="16">
         <v>368131.0</v>
       </c>
-      <c r="AE118" s="18">
+      <c r="AE118" s="19">
         <v>46241.0</v>
       </c>
-      <c r="AF118" s="15">
+      <c r="AF118" s="16">
         <v>4.0</v>
       </c>
-      <c r="AG118" s="15" t="s">
+      <c r="AG118" s="16" t="s">
         <v>831</v>
       </c>
-      <c r="AH118" s="19" t="s">
+      <c r="AH118" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="AI118" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ118" s="15" t="s">
+      <c r="AI118" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ118" s="16" t="s">
         <v>833</v>
       </c>
-      <c r="AK118" s="19" t="s">
+      <c r="AK118" s="20" t="s">
         <v>834</v>
       </c>
-      <c r="AL118" s="20"/>
-      <c r="AM118" s="20"/>
-      <c r="AN118" s="20"/>
-      <c r="AO118" s="20"/>
-      <c r="AP118" s="20"/>
-      <c r="AQ118" s="20"/>
-      <c r="AR118" s="20"/>
-      <c r="AS118" s="20"/>
-      <c r="AT118" s="20"/>
-      <c r="AU118" s="20"/>
-      <c r="AV118" s="21"/>
-      <c r="AW118" s="21"/>
-      <c r="AX118" s="21"/>
-      <c r="AY118" s="21"/>
-      <c r="AZ118" s="21"/>
-      <c r="BA118" s="21"/>
-      <c r="BB118" s="21"/>
-      <c r="BC118" s="21"/>
-      <c r="BD118" s="21"/>
+      <c r="AL118" s="21"/>
+      <c r="AM118" s="21"/>
+      <c r="AN118" s="21"/>
+      <c r="AO118" s="21"/>
+      <c r="AP118" s="21"/>
+      <c r="AQ118" s="21"/>
+      <c r="AR118" s="21"/>
+      <c r="AS118" s="21"/>
+      <c r="AT118" s="21"/>
+      <c r="AU118" s="21"/>
+      <c r="AV118" s="22"/>
+      <c r="AW118" s="22"/>
+      <c r="AX118" s="22"/>
+      <c r="AY118" s="22"/>
+      <c r="AZ118" s="22"/>
+      <c r="BA118" s="22"/>
+      <c r="BB118" s="22"/>
+      <c r="BC118" s="22"/>
+      <c r="BD118" s="22"/>
     </row>
     <row r="119">
-      <c r="A119" s="15">
+      <c r="A119" s="16">
         <v>96.0</v>
       </c>
-      <c r="B119" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C119" s="15" t="s">
+      <c r="B119" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C119" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="D119" s="16">
+      <c r="D119" s="17">
         <v>46174.04574074074</v>
       </c>
-      <c r="E119" s="15" t="s">
+      <c r="E119" s="16" t="s">
         <v>835</v>
       </c>
-      <c r="F119" s="15" t="b">
+      <c r="F119" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G119" s="15" t="s">
+      <c r="G119" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H119" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I119" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J119" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K119" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L119" s="15" t="s">
+      <c r="H119" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I119" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J119" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K119" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L119" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M119" s="17" t="s">
+      <c r="M119" s="18" t="s">
         <v>836</v>
       </c>
-      <c r="N119" s="16">
+      <c r="N119" s="17">
         <v>46174.04902777778</v>
       </c>
-      <c r="O119" s="15" t="s">
+      <c r="O119" s="16" t="s">
         <v>837</v>
       </c>
-      <c r="P119" s="15">
+      <c r="P119" s="16">
         <v>7.49252063445077E14</v>
       </c>
-      <c r="Q119" s="15" t="s">
+      <c r="Q119" s="16" t="s">
         <v>838</v>
       </c>
-      <c r="R119" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S119" s="15" t="s">
+      <c r="R119" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S119" s="16" t="s">
         <v>839</v>
       </c>
-      <c r="T119" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U119" s="15">
+      <c r="T119" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U119" s="16">
         <v>518.0</v>
       </c>
-      <c r="V119" s="15">
+      <c r="V119" s="16">
         <v>0.0</v>
       </c>
-      <c r="W119" s="15">
+      <c r="W119" s="16">
         <v>4570.0</v>
       </c>
-      <c r="X119" s="15">
+      <c r="X119" s="16">
         <v>3575.0</v>
       </c>
-      <c r="Y119" s="15">
+      <c r="Y119" s="16">
         <v>2753.0</v>
       </c>
-      <c r="Z119" s="15">
+      <c r="Z119" s="16">
         <v>169.0</v>
       </c>
-      <c r="AA119" s="15">
+      <c r="AA119" s="16">
         <v>7056.0</v>
       </c>
-      <c r="AB119" s="15">
+      <c r="AB119" s="16">
         <v>11.0</v>
       </c>
-      <c r="AC119" s="15">
+      <c r="AC119" s="16">
         <v>248.0</v>
       </c>
-      <c r="AD119" s="15">
+      <c r="AD119" s="16">
         <v>306900.0</v>
       </c>
-      <c r="AE119" s="18">
+      <c r="AE119" s="19">
         <v>46237.0</v>
       </c>
-      <c r="AF119" s="15">
+      <c r="AF119" s="16">
         <v>30.0</v>
       </c>
-      <c r="AG119" s="15">
+      <c r="AG119" s="16">
         <v>7.49252063445077E14</v>
       </c>
-      <c r="AH119" s="19" t="s">
+      <c r="AH119" s="20" t="s">
         <v>838</v>
       </c>
-      <c r="AI119" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ119" s="15" t="s">
+      <c r="AI119" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ119" s="16" t="s">
         <v>839</v>
       </c>
-      <c r="AK119" s="19" t="s">
+      <c r="AK119" s="20" t="s">
         <v>840</v>
       </c>
-      <c r="AL119" s="20"/>
-      <c r="AM119" s="20"/>
-      <c r="AN119" s="20"/>
-      <c r="AO119" s="20"/>
-      <c r="AP119" s="20"/>
-      <c r="AQ119" s="20"/>
-      <c r="AR119" s="20"/>
-      <c r="AS119" s="20"/>
-      <c r="AT119" s="20"/>
-      <c r="AU119" s="20"/>
-      <c r="AV119" s="21"/>
-      <c r="AW119" s="21"/>
-      <c r="AX119" s="21"/>
-      <c r="AY119" s="21"/>
-      <c r="AZ119" s="21"/>
-      <c r="BA119" s="21"/>
-      <c r="BB119" s="21"/>
-      <c r="BC119" s="21"/>
-      <c r="BD119" s="21"/>
+      <c r="AL119" s="21"/>
+      <c r="AM119" s="21"/>
+      <c r="AN119" s="21"/>
+      <c r="AO119" s="21"/>
+      <c r="AP119" s="21"/>
+      <c r="AQ119" s="21"/>
+      <c r="AR119" s="21"/>
+      <c r="AS119" s="21"/>
+      <c r="AT119" s="21"/>
+      <c r="AU119" s="21"/>
+      <c r="AV119" s="22"/>
+      <c r="AW119" s="22"/>
+      <c r="AX119" s="22"/>
+      <c r="AY119" s="22"/>
+      <c r="AZ119" s="22"/>
+      <c r="BA119" s="22"/>
+      <c r="BB119" s="22"/>
+      <c r="BC119" s="22"/>
+      <c r="BD119" s="22"/>
     </row>
     <row r="120">
-      <c r="A120" s="15">
+      <c r="A120" s="16">
         <v>97.0</v>
       </c>
-      <c r="B120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C120" s="15" t="s">
+      <c r="B120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C120" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="D120" s="16">
+      <c r="D120" s="17">
         <v>46174.129016203704</v>
       </c>
-      <c r="E120" s="15" t="s">
+      <c r="E120" s="16" t="s">
         <v>841</v>
       </c>
-      <c r="F120" s="15" t="b">
+      <c r="F120" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G120" s="15" t="s">
+      <c r="G120" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L120" s="15" t="s">
+      <c r="H120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L120" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M120" s="17" t="s">
+      <c r="M120" s="18" t="s">
         <v>842</v>
       </c>
-      <c r="N120" s="16">
+      <c r="N120" s="17">
         <v>46174.99594907407</v>
       </c>
-      <c r="O120" s="15" t="s">
+      <c r="O120" s="16" t="s">
         <v>843</v>
       </c>
-      <c r="P120" s="15">
+      <c r="P120" s="16">
         <v>7.96893052888034E14</v>
       </c>
-      <c r="Q120" s="15" t="s">
+      <c r="Q120" s="16" t="s">
         <v>844</v>
       </c>
-      <c r="R120" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="T120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U120" s="15">
+      <c r="R120" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="T120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U120" s="16">
         <v>1.0</v>
       </c>
-      <c r="V120" s="15">
+      <c r="V120" s="16">
         <v>0.0</v>
       </c>
-      <c r="W120" s="15">
+      <c r="W120" s="16">
         <v>228.0</v>
       </c>
-      <c r="X120" s="15">
+      <c r="X120" s="16">
         <v>2.0</v>
       </c>
-      <c r="Y120" s="15">
+      <c r="Y120" s="16">
         <v>4999.0</v>
       </c>
-      <c r="Z120" s="15">
+      <c r="Z120" s="16">
         <v>1892.0</v>
       </c>
-      <c r="AA120" s="15">
+      <c r="AA120" s="16">
         <v>6894.0</v>
       </c>
-      <c r="AB120" s="15">
+      <c r="AB120" s="16">
         <v>0.0</v>
       </c>
-      <c r="AC120" s="15">
+      <c r="AC120" s="16">
         <v>5.0</v>
       </c>
-      <c r="AD120" s="15">
+      <c r="AD120" s="16">
         <v>150292.0</v>
       </c>
-      <c r="AE120" s="18">
+      <c r="AE120" s="19">
         <v>46238.0</v>
       </c>
-      <c r="AF120" s="15">
+      <c r="AF120" s="16">
         <v>0.0</v>
       </c>
-      <c r="AG120" s="15" t="s">
+      <c r="AG120" s="16" t="s">
         <v>845</v>
       </c>
-      <c r="AH120" s="19" t="s">
+      <c r="AH120" s="20" t="s">
         <v>846</v>
       </c>
-      <c r="AI120" s="15" t="s">
+      <c r="AI120" s="16" t="s">
         <v>847</v>
       </c>
-      <c r="AJ120" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="AK120" s="19" t="s">
+      <c r="AJ120" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="AK120" s="20" t="s">
         <v>848</v>
       </c>
-      <c r="AL120" s="20"/>
-      <c r="AM120" s="20"/>
-      <c r="AN120" s="20"/>
-      <c r="AO120" s="20"/>
-      <c r="AP120" s="20"/>
-      <c r="AQ120" s="20"/>
-      <c r="AR120" s="20"/>
-      <c r="AS120" s="20"/>
-      <c r="AT120" s="20"/>
-      <c r="AU120" s="20"/>
-      <c r="AV120" s="21"/>
-      <c r="AW120" s="21"/>
-      <c r="AX120" s="21"/>
-      <c r="AY120" s="21"/>
-      <c r="AZ120" s="21"/>
-      <c r="BA120" s="21"/>
-      <c r="BB120" s="21"/>
-      <c r="BC120" s="21"/>
-      <c r="BD120" s="21"/>
+      <c r="AL120" s="21"/>
+      <c r="AM120" s="21"/>
+      <c r="AN120" s="21"/>
+      <c r="AO120" s="21"/>
+      <c r="AP120" s="21"/>
+      <c r="AQ120" s="21"/>
+      <c r="AR120" s="21"/>
+      <c r="AS120" s="21"/>
+      <c r="AT120" s="21"/>
+      <c r="AU120" s="21"/>
+      <c r="AV120" s="22"/>
+      <c r="AW120" s="22"/>
+      <c r="AX120" s="22"/>
+      <c r="AY120" s="22"/>
+      <c r="AZ120" s="22"/>
+      <c r="BA120" s="22"/>
+      <c r="BB120" s="22"/>
+      <c r="BC120" s="22"/>
+      <c r="BD120" s="22"/>
     </row>
     <row r="121">
-      <c r="A121" s="15">
+      <c r="A121" s="16">
         <v>108.0</v>
       </c>
-      <c r="B121" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C121" s="15" t="s">
+      <c r="B121" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C121" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="D121" s="16">
+      <c r="D121" s="17">
         <v>46174.02142361111</v>
       </c>
-      <c r="E121" s="15" t="s">
+      <c r="E121" s="16" t="s">
         <v>849</v>
       </c>
-      <c r="F121" s="15" t="b">
+      <c r="F121" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="G121" s="15" t="s">
+      <c r="G121" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H121" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I121" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J121" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="K121" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="L121" s="15" t="s">
+      <c r="H121" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I121" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J121" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K121" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L121" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M121" s="17" t="s">
+      <c r="M121" s="18" t="s">
         <v>850</v>
       </c>
-      <c r="N121" s="16">
+      <c r="N121" s="17">
         <v>46174.03134259259</v>
       </c>
-      <c r="O121" s="15" t="s">
+      <c r="O121" s="16" t="s">
         <v>851</v>
       </c>
-      <c r="P121" s="15">
+      <c r="P121" s="16">
         <v>3.69279539472281E14</v>
       </c>
-      <c r="Q121" s="15" t="s">
+      <c r="Q121" s="16" t="s">
         <v>852</v>
       </c>
-      <c r="R121" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="S121" s="15" t="s">
+      <c r="R121" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="S121" s="16" t="s">
         <v>853</v>
       </c>
-      <c r="T121" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="U121" s="15">
+      <c r="T121" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="U121" s="16">
         <v>105.0</v>
       </c>
-      <c r="V121" s="15">
+      <c r="V121" s="16">
         <v>0.0</v>
       </c>
-      <c r="W121" s="15">
+      <c r="W121" s="16">
         <v>3430.0</v>
       </c>
-      <c r="X121" s="15">
+      <c r="X121" s="16">
         <v>2183.0</v>
       </c>
-      <c r="Y121" s="15">
+      <c r="Y121" s="16">
         <v>3523.0</v>
       </c>
-      <c r="Z121" s="15">
+      <c r="Z121" s="16">
         <v>182.0</v>
       </c>
-      <c r="AA121" s="15">
+      <c r="AA121" s="16">
         <v>6110.0</v>
       </c>
-      <c r="AB121" s="15">
+      <c r="AB121" s="16">
         <v>66.0</v>
       </c>
-      <c r="AC121" s="15">
+      <c r="AC121" s="16">
         <v>477.0</v>
       </c>
-      <c r="AD121" s="15">
+      <c r="AD121" s="16">
         <v>430510.0</v>
       </c>
-      <c r="AE121" s="18">
+      <c r="AE121" s="19">
         <v>46237.0</v>
       </c>
-      <c r="AF121" s="15">
+      <c r="AF121" s="16">
         <v>51.0</v>
       </c>
-      <c r="AG121" s="15">
+      <c r="AG121" s="16">
         <v>3.69279539472281E14</v>
       </c>
-      <c r="AH121" s="19" t="s">
+      <c r="AH121" s="20" t="s">
         <v>852</v>
       </c>
-      <c r="AI121" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ121" s="15" t="s">
+      <c r="AI121" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ121" s="16" t="s">
         <v>853</v>
       </c>
-      <c r="AK121" s="19" t="s">
+      <c r="AK121" s="20" t="s">
         <v>854</v>
       </c>
-      <c r="AL121" s="20"/>
-      <c r="AM121" s="20"/>
-      <c r="AN121" s="20"/>
-      <c r="AO121" s="20"/>
-      <c r="AP121" s="20"/>
-      <c r="AQ121" s="20"/>
-      <c r="AR121" s="20"/>
-      <c r="AS121" s="20"/>
-      <c r="AT121" s="20"/>
-      <c r="AU121" s="20"/>
-      <c r="AV121" s="21"/>
-      <c r="AW121" s="21"/>
-      <c r="AX121" s="21"/>
-      <c r="AY121" s="21"/>
-      <c r="AZ121" s="21"/>
-      <c r="BA121" s="21"/>
-      <c r="BB121" s="21"/>
-      <c r="BC121" s="21"/>
-      <c r="BD121" s="21"/>
+      <c r="AL121" s="21"/>
+      <c r="AM121" s="21"/>
+      <c r="AN121" s="21"/>
+      <c r="AO121" s="21"/>
+      <c r="AP121" s="21"/>
+      <c r="AQ121" s="21"/>
+      <c r="AR121" s="21"/>
+      <c r="AS121" s="21"/>
+      <c r="AT121" s="21"/>
+      <c r="AU121" s="21"/>
+      <c r="AV121" s="22"/>
+      <c r="AW121" s="22"/>
+      <c r="AX121" s="22"/>
+      <c r="AY121" s="22"/>
+      <c r="AZ121" s="22"/>
+      <c r="BA121" s="22"/>
+      <c r="BB121" s="22"/>
+      <c r="BC121" s="22"/>
+      <c r="BD121" s="22"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>